<commit_message>
feat(epp): auto fecha_cambio +6 meses, logo BV embebido, fitToPage 1x1
- epps_core: _add_months helper, fecha_cambio default = fecha_entrega + 6 meses si no se proporciona
- template epp_template.xlsx: logo Bureau Veritas embebido en A1 (110x80 px), page setup fitToPage 1 ancho x 1 alto, portrait A4, margins reducidos, print area A1:I34
- Includes templates/logo_bureau_veritas.jpg

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/epp_template.xlsx
+++ b/templates/epp_template.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F-004" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'F-004'!$A$1:$I$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'F-004'!$A$1:$I$34</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -472,94 +472,31 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
+  <oneCellAnchor>
     <from>
       <col>0</col>
-      <colOff>330200</colOff>
+      <colOff>0</colOff>
       <row>0</row>
-      <rowOff>88900</rowOff>
+      <rowOff>0</rowOff>
     </from>
-    <to>
-      <col>0</col>
-      <colOff>977900</colOff>
-      <row>2</row>
-      <rowOff>273050</rowOff>
-    </to>
+    <ext cx="1047750" cy="762000"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="2" name="Imagen 1"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="330200" y="88900"/>
-          <a:ext cx="647700" cy="831850"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>6</col>
-      <colOff>488950</colOff>
-      <row>4</row>
-      <rowOff>50800</rowOff>
-    </from>
-    <to>
-      <col>8</col>
-      <colOff>577850</colOff>
-      <row>8</row>
-      <rowOff>254000</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Imagen 2"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="7124700" y="1206500"/>
-          <a:ext cx="1993900" cy="1905000"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -883,9 +820,9 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col width="36.90625" customWidth="1" min="1" max="1"/>
@@ -1870,8 +1807,8 @@
     <mergeCell ref="G23:I23"/>
     <mergeCell ref="G17:I17"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="55"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="55" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;C&amp;"Aptos"&amp;11 &amp;K000000_x000d_# BV_C2_Internal</oddFooter>

</xml_diff>